<commit_message>
test: add comprehensive end-to-end verification script and verify all admin/evaluator workflows
</commit_message>
<xml_diff>
--- a/data/2026_test.xlsx
+++ b/data/2026_test.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="102">
   <si>
     <t>연번</t>
   </si>
@@ -109,12 +109,6 @@
     <t>기술5급</t>
   </si>
   <si>
-    <t>개발사업본부</t>
-  </si>
-  <si>
-    <t>사업계획처</t>
-  </si>
-  <si>
     <t>지역상생</t>
   </si>
   <si>
@@ -187,24 +181,12 @@
     <t>[자유제안] 음주운전 점검방식 개선으로 개인정보 유출 리스크 차단</t>
   </si>
   <si>
-    <t>9</t>
-  </si>
-  <si>
-    <t>오석현</t>
-  </si>
-  <si>
     <t>재무부</t>
   </si>
   <si>
     <t>경영지원실 재무부</t>
   </si>
   <si>
-    <t>2026-07-30 13:14:00</t>
-  </si>
-  <si>
-    <t>[지정제안]물가·적산정보 통합패키지 구매 및 예산편성 기준 일원화</t>
-  </si>
-  <si>
     <t>공원수련관관리처</t>
   </si>
   <si>
@@ -214,12 +196,6 @@
     <t>시설관리처</t>
   </si>
   <si>
-    <t>시설운영부</t>
-  </si>
-  <si>
-    <t>시설관리처 시설운영부</t>
-  </si>
-  <si>
     <t>김재범</t>
   </si>
   <si>
@@ -232,18 +208,6 @@
     <t>시민회관체육운영처 여가체육부</t>
   </si>
   <si>
-    <t>총무행정부</t>
-  </si>
-  <si>
-    <t>경영지원실 총무행정부</t>
-  </si>
-  <si>
-    <t>인사부</t>
-  </si>
-  <si>
-    <t>경영지원실 인사부</t>
-  </si>
-  <si>
     <t>스마트정보부</t>
   </si>
   <si>
@@ -253,9 +217,6 @@
     <t>안전</t>
   </si>
   <si>
-    <t>김일권</t>
-  </si>
-  <si>
     <t>주차관리부</t>
   </si>
   <si>
@@ -304,81 +265,15 @@
     <t>[자유제안] 엘리베이터 층별 안내 스티커 부착</t>
   </si>
   <si>
-    <t>26</t>
-  </si>
-  <si>
-    <t>2026-08-04 11:32:00</t>
-  </si>
-  <si>
-    <t>과천도시공사 비정규직관리지침 개정 요청</t>
-  </si>
-  <si>
     <t>시설지원부</t>
   </si>
   <si>
     <t>공원수련관관리처 시설지원부</t>
   </si>
   <si>
-    <t>안전총괄단</t>
-  </si>
-  <si>
-    <t>AI혁신</t>
-  </si>
-  <si>
-    <t>최성호</t>
-  </si>
-  <si>
-    <t>41</t>
-  </si>
-  <si>
-    <t>황광엽</t>
-  </si>
-  <si>
-    <t>판매·보상부</t>
-  </si>
-  <si>
-    <t>사업계획처 판매·보상부</t>
-  </si>
-  <si>
-    <t>2026-08-13 09:45:00</t>
-  </si>
-  <si>
-    <t>(실행제안)과천과천 공공주택지구 이주촉진 및 현장관리 전문지원체계 구축</t>
-  </si>
-  <si>
-    <t>42</t>
-  </si>
-  <si>
     <t>시설개선</t>
   </si>
   <si>
-    <t>2026-08-13 09:48:00</t>
-  </si>
-  <si>
-    <t>[실행제안] 관문체육공원 고사 느티나무 하부 녹지대 경관 정원 조성</t>
-  </si>
-  <si>
-    <t>43</t>
-  </si>
-  <si>
-    <t>2026-08-13 09:51:00</t>
-  </si>
-  <si>
-    <t>[실행제안] 관문체육공원 녹지대 저관리형 정원 조성</t>
-  </si>
-  <si>
-    <t>44</t>
-  </si>
-  <si>
-    <t>김혜경</t>
-  </si>
-  <si>
-    <t>2026-08-13 11:28:00</t>
-  </si>
-  <si>
-    <t>[지정제안] AI 기반 사규 개정업무 업무혁신</t>
-  </si>
-  <si>
     <t>59</t>
   </si>
   <si>
@@ -406,24 +301,6 @@
     <t>(자유제안) 화장실 위생 개선 및 노로바이러스 감염 예방을 위한 양변기 손잡이 설치</t>
   </si>
   <si>
-    <t>64</t>
-  </si>
-  <si>
-    <t>김동규</t>
-  </si>
-  <si>
-    <t>안전사고 예방</t>
-  </si>
-  <si>
-    <t>2026-08-24 18:33:00</t>
-  </si>
-  <si>
-    <t>[지정제안] 시민회관 볼판 승강기 교체를 통한 안전사고 예방</t>
-  </si>
-  <si>
-    <t>성화진</t>
-  </si>
-  <si>
     <t>143</t>
   </si>
   <si>
@@ -443,15 +320,6 @@
   </si>
   <si>
     <t>장애인 주차구역 스마트단속시스템</t>
-  </si>
-  <si>
-    <t>147</t>
-  </si>
-  <si>
-    <t>2026-10-01 10:18:00</t>
-  </si>
-  <si>
-    <t>사원증 QR을 활용한 디지털 명함 도입 및 종이명함 제작 최소화</t>
   </si>
 </sst>
 </file>
@@ -832,7 +700,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R18"/>
+  <dimension ref="A1:R10"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.77734375" customWidth="1"/>
@@ -970,49 +838,49 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D3" t="s">
         <v>34</v>
       </c>
-      <c r="C3" t="s">
+      <c r="E3" t="s">
         <v>35</v>
       </c>
-      <c r="D3" t="s">
+      <c r="F3" t="s">
         <v>36</v>
       </c>
-      <c r="E3" t="s">
+      <c r="G3" t="s">
         <v>37</v>
       </c>
-      <c r="F3" t="s">
+      <c r="H3" t="s">
         <v>38</v>
       </c>
-      <c r="G3" t="s">
+      <c r="I3" t="s">
         <v>39</v>
       </c>
-      <c r="H3" t="s">
+      <c r="J3" t="s">
         <v>40</v>
       </c>
-      <c r="I3" t="s">
+      <c r="K3" t="s">
+        <v>35</v>
+      </c>
+      <c r="L3" t="s">
+        <v>36</v>
+      </c>
+      <c r="M3" t="s">
+        <v>37</v>
+      </c>
+      <c r="N3" t="s">
         <v>41</v>
       </c>
-      <c r="J3" t="s">
+      <c r="O3" t="s">
         <v>42</v>
       </c>
-      <c r="K3" t="s">
-        <v>37</v>
-      </c>
-      <c r="L3" t="s">
-        <v>38</v>
-      </c>
-      <c r="M3" t="s">
-        <v>39</v>
-      </c>
-      <c r="N3" t="s">
+      <c r="P3" t="s">
         <v>43</v>
-      </c>
-      <c r="O3" t="s">
-        <v>44</v>
-      </c>
-      <c r="P3" t="s">
-        <v>45</v>
       </c>
       <c r="Q3" t="s">
         <v>29</v>
@@ -1026,10 +894,10 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D4" t="s">
         <v>20</v>
@@ -1038,37 +906,37 @@
         <v>21</v>
       </c>
       <c r="F4" t="s">
+        <v>46</v>
+      </c>
+      <c r="G4" t="s">
+        <v>47</v>
+      </c>
+      <c r="H4" t="s">
         <v>48</v>
       </c>
-      <c r="G4" t="s">
+      <c r="I4" t="s">
         <v>49</v>
       </c>
-      <c r="H4" t="s">
+      <c r="J4" t="s">
         <v>50</v>
       </c>
-      <c r="I4" t="s">
+      <c r="K4" t="s">
         <v>51</v>
       </c>
-      <c r="J4" t="s">
+      <c r="L4" t="s">
         <v>52</v>
       </c>
-      <c r="K4" t="s">
+      <c r="M4" t="s">
+        <v>52</v>
+      </c>
+      <c r="N4" t="s">
+        <v>52</v>
+      </c>
+      <c r="O4" t="s">
         <v>53</v>
       </c>
-      <c r="L4" t="s">
+      <c r="P4" t="s">
         <v>54</v>
-      </c>
-      <c r="M4" t="s">
-        <v>54</v>
-      </c>
-      <c r="N4" t="s">
-        <v>54</v>
-      </c>
-      <c r="O4" t="s">
-        <v>55</v>
-      </c>
-      <c r="P4" t="s">
-        <v>56</v>
       </c>
       <c r="Q4" t="s">
         <v>29</v>
@@ -1079,52 +947,52 @@
     </row>
     <row r="5" spans="1:18" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="B5" t="s">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="C5" t="s">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="D5" t="s">
-        <v>30</v>
+        <v>71</v>
       </c>
       <c r="E5" t="s">
-        <v>53</v>
+        <v>35</v>
       </c>
       <c r="F5" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G5" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="H5" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="I5" t="s">
         <v>25</v>
       </c>
       <c r="J5" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="K5" t="s">
         <v>21</v>
       </c>
       <c r="L5" t="s">
-        <v>22</v>
+        <v>46</v>
       </c>
       <c r="M5" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="N5" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="O5" t="s">
-        <v>61</v>
+        <v>72</v>
       </c>
       <c r="P5" t="s">
-        <v>62</v>
+        <v>73</v>
       </c>
       <c r="Q5" t="s">
         <v>29</v>
@@ -1135,52 +1003,52 @@
     </row>
     <row r="6" spans="1:18" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B6" t="s">
+        <v>78</v>
+      </c>
+      <c r="C6" t="s">
+        <v>76</v>
+      </c>
+      <c r="D6" t="s">
+        <v>77</v>
+      </c>
+      <c r="E6" t="s">
+        <v>35</v>
+      </c>
+      <c r="F6" t="s">
+        <v>36</v>
+      </c>
+      <c r="G6" t="s">
+        <v>37</v>
+      </c>
+      <c r="H6" t="s">
+        <v>41</v>
+      </c>
+      <c r="I6" t="s">
+        <v>49</v>
+      </c>
+      <c r="J6" t="s">
+        <v>58</v>
+      </c>
+      <c r="K6" t="s">
+        <v>35</v>
+      </c>
+      <c r="L6" t="s">
+        <v>59</v>
+      </c>
+      <c r="M6" t="s">
+        <v>79</v>
+      </c>
+      <c r="N6" t="s">
+        <v>80</v>
+      </c>
+      <c r="O6" t="s">
+        <v>81</v>
+      </c>
+      <c r="P6" t="s">
         <v>82</v>
-      </c>
-      <c r="C6" t="s">
-        <v>83</v>
-      </c>
-      <c r="D6" t="s">
-        <v>84</v>
-      </c>
-      <c r="E6" t="s">
-        <v>37</v>
-      </c>
-      <c r="F6" t="s">
-        <v>65</v>
-      </c>
-      <c r="G6" t="s">
-        <v>80</v>
-      </c>
-      <c r="H6" t="s">
-        <v>81</v>
-      </c>
-      <c r="I6" t="s">
-        <v>25</v>
-      </c>
-      <c r="J6" t="s">
-        <v>42</v>
-      </c>
-      <c r="K6" t="s">
-        <v>21</v>
-      </c>
-      <c r="L6" t="s">
-        <v>48</v>
-      </c>
-      <c r="M6" t="s">
-        <v>76</v>
-      </c>
-      <c r="N6" t="s">
-        <v>77</v>
-      </c>
-      <c r="O6" t="s">
-        <v>85</v>
-      </c>
-      <c r="P6" t="s">
-        <v>86</v>
       </c>
       <c r="Q6" t="s">
         <v>29</v>
@@ -1191,52 +1059,52 @@
     </row>
     <row r="7" spans="1:18" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>19</v>
+        <v>52</v>
       </c>
       <c r="B7" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="C7" t="s">
+        <v>87</v>
+      </c>
+      <c r="D7" t="s">
+        <v>71</v>
+      </c>
+      <c r="E7" t="s">
+        <v>21</v>
+      </c>
+      <c r="F7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G7" t="s">
+        <v>55</v>
+      </c>
+      <c r="H7" t="s">
+        <v>56</v>
+      </c>
+      <c r="I7" t="s">
+        <v>25</v>
+      </c>
+      <c r="J7" t="s">
+        <v>31</v>
+      </c>
+      <c r="K7" t="s">
+        <v>21</v>
+      </c>
+      <c r="L7" t="s">
+        <v>22</v>
+      </c>
+      <c r="M7" t="s">
+        <v>55</v>
+      </c>
+      <c r="N7" t="s">
+        <v>56</v>
+      </c>
+      <c r="O7" t="s">
+        <v>88</v>
+      </c>
+      <c r="P7" t="s">
         <v>89</v>
-      </c>
-      <c r="D7" t="s">
-        <v>90</v>
-      </c>
-      <c r="E7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F7" t="s">
-        <v>38</v>
-      </c>
-      <c r="G7" t="s">
-        <v>39</v>
-      </c>
-      <c r="H7" t="s">
-        <v>43</v>
-      </c>
-      <c r="I7" t="s">
-        <v>51</v>
-      </c>
-      <c r="J7" t="s">
-        <v>64</v>
-      </c>
-      <c r="K7" t="s">
-        <v>37</v>
-      </c>
-      <c r="L7" t="s">
-        <v>65</v>
-      </c>
-      <c r="M7" t="s">
-        <v>92</v>
-      </c>
-      <c r="N7" t="s">
-        <v>93</v>
-      </c>
-      <c r="O7" t="s">
-        <v>94</v>
-      </c>
-      <c r="P7" t="s">
-        <v>95</v>
       </c>
       <c r="Q7" t="s">
         <v>29</v>
@@ -1247,52 +1115,52 @@
     </row>
     <row r="8" spans="1:18" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>20</v>
+        <v>54</v>
       </c>
       <c r="B8" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="C8" t="s">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="D8" t="s">
-        <v>36</v>
+        <v>92</v>
       </c>
       <c r="E8" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F8" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="G8" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="H8" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="I8" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="J8" t="s">
-        <v>52</v>
+        <v>66</v>
       </c>
       <c r="K8" t="s">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="L8" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="M8" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="N8" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="O8" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="P8" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="Q8" t="s">
         <v>29</v>
@@ -1303,52 +1171,52 @@
     </row>
     <row r="9" spans="1:18" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>34</v>
+        <v>134</v>
       </c>
       <c r="B9" t="s">
-        <v>104</v>
+        <v>95</v>
       </c>
       <c r="C9" t="s">
-        <v>105</v>
+        <v>96</v>
       </c>
       <c r="D9" t="s">
-        <v>69</v>
+        <v>30</v>
       </c>
       <c r="E9" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="F9" t="s">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="G9" t="s">
-        <v>106</v>
+        <v>74</v>
       </c>
       <c r="H9" t="s">
-        <v>107</v>
+        <v>75</v>
       </c>
       <c r="I9" t="s">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="J9" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="K9" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="L9" t="s">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="M9" t="s">
-        <v>106</v>
+        <v>74</v>
       </c>
       <c r="N9" t="s">
-        <v>107</v>
+        <v>75</v>
       </c>
       <c r="O9" t="s">
-        <v>108</v>
+        <v>97</v>
       </c>
       <c r="P9" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="Q9" t="s">
         <v>29</v>
@@ -1359,505 +1227,57 @@
     </row>
     <row r="10" spans="1:18" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A10">
+        <v>136</v>
+      </c>
+      <c r="B10" t="s">
+        <v>99</v>
+      </c>
+      <c r="C10" t="s">
+        <v>60</v>
+      </c>
+      <c r="D10" t="s">
+        <v>61</v>
+      </c>
+      <c r="E10" t="s">
         <v>35</v>
       </c>
-      <c r="B10" t="s">
-        <v>110</v>
-      </c>
-      <c r="C10" t="s">
-        <v>103</v>
-      </c>
-      <c r="D10" t="s">
-        <v>30</v>
-      </c>
-      <c r="E10" t="s">
-        <v>37</v>
-      </c>
       <c r="F10" t="s">
+        <v>36</v>
+      </c>
+      <c r="G10" t="s">
+        <v>62</v>
+      </c>
+      <c r="H10" t="s">
         <v>63</v>
       </c>
-      <c r="G10" t="s">
-        <v>99</v>
-      </c>
-      <c r="H10" t="s">
+      <c r="I10" t="s">
+        <v>49</v>
+      </c>
+      <c r="J10" t="s">
+        <v>85</v>
+      </c>
+      <c r="K10" t="s">
+        <v>35</v>
+      </c>
+      <c r="L10" t="s">
+        <v>57</v>
+      </c>
+      <c r="M10" t="s">
+        <v>83</v>
+      </c>
+      <c r="N10" t="s">
+        <v>84</v>
+      </c>
+      <c r="O10" t="s">
         <v>100</v>
       </c>
-      <c r="I10" t="s">
-        <v>41</v>
-      </c>
-      <c r="J10" t="s">
-        <v>111</v>
-      </c>
-      <c r="K10" t="s">
-        <v>37</v>
-      </c>
-      <c r="L10" t="s">
-        <v>63</v>
-      </c>
-      <c r="M10" t="s">
-        <v>99</v>
-      </c>
-      <c r="N10" t="s">
-        <v>100</v>
-      </c>
-      <c r="O10" t="s">
-        <v>112</v>
-      </c>
       <c r="P10" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="Q10" t="s">
         <v>29</v>
       </c>
       <c r="R10" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="11" spans="1:18" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A11">
-        <v>36</v>
-      </c>
-      <c r="B11" t="s">
-        <v>114</v>
-      </c>
-      <c r="C11" t="s">
-        <v>103</v>
-      </c>
-      <c r="D11" t="s">
-        <v>30</v>
-      </c>
-      <c r="E11" t="s">
-        <v>37</v>
-      </c>
-      <c r="F11" t="s">
-        <v>63</v>
-      </c>
-      <c r="G11" t="s">
-        <v>99</v>
-      </c>
-      <c r="H11" t="s">
-        <v>100</v>
-      </c>
-      <c r="I11" t="s">
-        <v>41</v>
-      </c>
-      <c r="J11" t="s">
-        <v>111</v>
-      </c>
-      <c r="K11" t="s">
-        <v>37</v>
-      </c>
-      <c r="L11" t="s">
-        <v>63</v>
-      </c>
-      <c r="M11" t="s">
-        <v>99</v>
-      </c>
-      <c r="N11" t="s">
-        <v>100</v>
-      </c>
-      <c r="O11" t="s">
-        <v>115</v>
-      </c>
-      <c r="P11" t="s">
-        <v>116</v>
-      </c>
-      <c r="Q11" t="s">
-        <v>29</v>
-      </c>
-      <c r="R11" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="12" spans="1:18" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A12">
-        <v>37</v>
-      </c>
-      <c r="B12" t="s">
-        <v>117</v>
-      </c>
-      <c r="C12" t="s">
-        <v>118</v>
-      </c>
-      <c r="D12" t="s">
-        <v>69</v>
-      </c>
-      <c r="E12" t="s">
-        <v>21</v>
-      </c>
-      <c r="F12" t="s">
-        <v>22</v>
-      </c>
-      <c r="G12" t="s">
-        <v>74</v>
-      </c>
-      <c r="H12" t="s">
-        <v>75</v>
-      </c>
-      <c r="I12" t="s">
-        <v>25</v>
-      </c>
-      <c r="J12" t="s">
-        <v>102</v>
-      </c>
-      <c r="K12" t="s">
-        <v>21</v>
-      </c>
-      <c r="L12" t="s">
-        <v>48</v>
-      </c>
-      <c r="M12" t="s">
-        <v>49</v>
-      </c>
-      <c r="N12" t="s">
-        <v>50</v>
-      </c>
-      <c r="O12" t="s">
-        <v>119</v>
-      </c>
-      <c r="P12" t="s">
-        <v>120</v>
-      </c>
-      <c r="Q12" t="s">
-        <v>29</v>
-      </c>
-      <c r="R12" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="13" spans="1:18" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A13">
-        <v>52</v>
-      </c>
-      <c r="B13" t="s">
-        <v>121</v>
-      </c>
-      <c r="C13" t="s">
-        <v>122</v>
-      </c>
-      <c r="D13" t="s">
-        <v>84</v>
-      </c>
-      <c r="E13" t="s">
-        <v>21</v>
-      </c>
-      <c r="F13" t="s">
-        <v>22</v>
-      </c>
-      <c r="G13" t="s">
-        <v>59</v>
-      </c>
-      <c r="H13" t="s">
-        <v>60</v>
-      </c>
-      <c r="I13" t="s">
-        <v>25</v>
-      </c>
-      <c r="J13" t="s">
-        <v>33</v>
-      </c>
-      <c r="K13" t="s">
-        <v>21</v>
-      </c>
-      <c r="L13" t="s">
-        <v>22</v>
-      </c>
-      <c r="M13" t="s">
-        <v>59</v>
-      </c>
-      <c r="N13" t="s">
-        <v>60</v>
-      </c>
-      <c r="O13" t="s">
-        <v>123</v>
-      </c>
-      <c r="P13" t="s">
-        <v>124</v>
-      </c>
-      <c r="Q13" t="s">
-        <v>29</v>
-      </c>
-      <c r="R13" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="14" spans="1:18" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A14">
-        <v>54</v>
-      </c>
-      <c r="B14" t="s">
-        <v>125</v>
-      </c>
-      <c r="C14" t="s">
-        <v>126</v>
-      </c>
-      <c r="D14" t="s">
-        <v>127</v>
-      </c>
-      <c r="E14" t="s">
-        <v>37</v>
-      </c>
-      <c r="F14" t="s">
-        <v>63</v>
-      </c>
-      <c r="G14" t="s">
-        <v>87</v>
-      </c>
-      <c r="H14" t="s">
-        <v>88</v>
-      </c>
-      <c r="I14" t="s">
-        <v>51</v>
-      </c>
-      <c r="J14" t="s">
-        <v>78</v>
-      </c>
-      <c r="K14" t="s">
-        <v>37</v>
-      </c>
-      <c r="L14" t="s">
-        <v>63</v>
-      </c>
-      <c r="M14" t="s">
-        <v>99</v>
-      </c>
-      <c r="N14" t="s">
-        <v>100</v>
-      </c>
-      <c r="O14" t="s">
-        <v>128</v>
-      </c>
-      <c r="P14" t="s">
-        <v>129</v>
-      </c>
-      <c r="Q14" t="s">
-        <v>29</v>
-      </c>
-      <c r="R14" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="15" spans="1:18" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A15">
-        <v>56</v>
-      </c>
-      <c r="B15" t="s">
-        <v>130</v>
-      </c>
-      <c r="C15" t="s">
-        <v>131</v>
-      </c>
-      <c r="D15" t="s">
-        <v>36</v>
-      </c>
-      <c r="E15" t="s">
-        <v>37</v>
-      </c>
-      <c r="F15" t="s">
-        <v>65</v>
-      </c>
-      <c r="G15" t="s">
-        <v>66</v>
-      </c>
-      <c r="H15" t="s">
-        <v>66</v>
-      </c>
-      <c r="I15" t="s">
-        <v>25</v>
-      </c>
-      <c r="J15" t="s">
-        <v>132</v>
-      </c>
-      <c r="K15" t="s">
-        <v>37</v>
-      </c>
-      <c r="L15" t="s">
-        <v>65</v>
-      </c>
-      <c r="M15" t="s">
-        <v>66</v>
-      </c>
-      <c r="N15" t="s">
-        <v>67</v>
-      </c>
-      <c r="O15" t="s">
-        <v>133</v>
-      </c>
-      <c r="P15" t="s">
-        <v>134</v>
-      </c>
-      <c r="Q15" t="s">
-        <v>29</v>
-      </c>
-      <c r="R15" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="16" spans="1:18" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A16">
-        <v>134</v>
-      </c>
-      <c r="B16" t="s">
-        <v>136</v>
-      </c>
-      <c r="C16" t="s">
-        <v>137</v>
-      </c>
-      <c r="D16" t="s">
-        <v>30</v>
-      </c>
-      <c r="E16" t="s">
-        <v>37</v>
-      </c>
-      <c r="F16" t="s">
-        <v>63</v>
-      </c>
-      <c r="G16" t="s">
-        <v>87</v>
-      </c>
-      <c r="H16" t="s">
-        <v>88</v>
-      </c>
-      <c r="I16" t="s">
-        <v>25</v>
-      </c>
-      <c r="J16" t="s">
-        <v>42</v>
-      </c>
-      <c r="K16" t="s">
-        <v>37</v>
-      </c>
-      <c r="L16" t="s">
-        <v>63</v>
-      </c>
-      <c r="M16" t="s">
-        <v>87</v>
-      </c>
-      <c r="N16" t="s">
-        <v>88</v>
-      </c>
-      <c r="O16" t="s">
-        <v>138</v>
-      </c>
-      <c r="P16" t="s">
-        <v>139</v>
-      </c>
-      <c r="Q16" t="s">
-        <v>29</v>
-      </c>
-      <c r="R16" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="17" spans="1:18" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A17">
-        <v>136</v>
-      </c>
-      <c r="B17" t="s">
-        <v>140</v>
-      </c>
-      <c r="C17" t="s">
-        <v>68</v>
-      </c>
-      <c r="D17" t="s">
-        <v>69</v>
-      </c>
-      <c r="E17" t="s">
-        <v>37</v>
-      </c>
-      <c r="F17" t="s">
-        <v>38</v>
-      </c>
-      <c r="G17" t="s">
-        <v>70</v>
-      </c>
-      <c r="H17" t="s">
-        <v>71</v>
-      </c>
-      <c r="I17" t="s">
-        <v>51</v>
-      </c>
-      <c r="J17" t="s">
-        <v>111</v>
-      </c>
-      <c r="K17" t="s">
-        <v>37</v>
-      </c>
-      <c r="L17" t="s">
-        <v>63</v>
-      </c>
-      <c r="M17" t="s">
-        <v>99</v>
-      </c>
-      <c r="N17" t="s">
-        <v>100</v>
-      </c>
-      <c r="O17" t="s">
-        <v>141</v>
-      </c>
-      <c r="P17" t="s">
-        <v>142</v>
-      </c>
-      <c r="Q17" t="s">
-        <v>29</v>
-      </c>
-      <c r="R17" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="18" spans="1:18" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A18">
-        <v>137</v>
-      </c>
-      <c r="B18" t="s">
-        <v>143</v>
-      </c>
-      <c r="C18" t="s">
-        <v>135</v>
-      </c>
-      <c r="D18" t="s">
-        <v>36</v>
-      </c>
-      <c r="E18" t="s">
-        <v>53</v>
-      </c>
-      <c r="F18" t="s">
-        <v>101</v>
-      </c>
-      <c r="G18" t="s">
-        <v>101</v>
-      </c>
-      <c r="H18" t="s">
-        <v>101</v>
-      </c>
-      <c r="I18" t="s">
-        <v>51</v>
-      </c>
-      <c r="J18" t="s">
-        <v>42</v>
-      </c>
-      <c r="K18" t="s">
-        <v>21</v>
-      </c>
-      <c r="L18" t="s">
-        <v>22</v>
-      </c>
-      <c r="M18" t="s">
-        <v>72</v>
-      </c>
-      <c r="N18" t="s">
-        <v>73</v>
-      </c>
-      <c r="O18" t="s">
-        <v>144</v>
-      </c>
-      <c r="P18" t="s">
-        <v>145</v>
-      </c>
-      <c r="Q18" t="s">
-        <v>29</v>
-      </c>
-      <c r="R18" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1866,7 +1286,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:R2 A3:R5 A6:R6 A9:R12 A16:R16 A13:R13 A7:R8 A14:R14 A17:R18 A15:R15" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:R2 A3:R4 A5:R5 A9:R9 A7:R7 A6:R6 A8:R8 A10:R10" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>